<commit_message>
feat: calendario talleres en email semanal + mejoras WooCommerce
- _seccion_talleres(): bloque HTML con proximos eventos en email del lunes
  (nombre, fecha, horario, plazas disponibles en color, precio)
- _limpiar_nombre_taller(): elimina fecha y sufijos 'Comestibles/Tasca Barea'
- generar_inventario_talleres(): ahora extrae stock_quantity, stock_status, precio
- _normalizar_pedidos_wc(): DataFrame 7 columnas limpias (antes ~69 de WC)
- talleres_programados.json: inventario actualizado de eventos
- cargar_historico_wc.py: script carga historico pedidos WooCommerce
- DiccionarioProveedoresCategoria.xlsx: actualizado
</commit_message>
<xml_diff>
--- a/datos/DiccionarioProveedoresCategoria.xlsx
+++ b/datos/DiccionarioProveedoresCategoria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_ARCHIVOS\TRABAJO\Facturas\gestion-facturas\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E8B69D-A27B-4182-AE62-9C075E141DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F26653E-1855-4FD7-A3BE-A40B27ED4F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4221" uniqueCount="1285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4251" uniqueCount="1297">
   <si>
     <t>PROVEEDOR</t>
   </si>
@@ -3904,6 +3904,42 @@
   </si>
   <si>
     <t>RUFINO</t>
+  </si>
+  <si>
+    <t>11071 = MOUSSE DE ALCACHOFA 30 u x 110g</t>
+  </si>
+  <si>
+    <t>11072 = MOUSSE QUESO CURADO/TRUFA NEGRA</t>
+  </si>
+  <si>
+    <t>DIL</t>
+  </si>
+  <si>
+    <t>11077 =PATE DE JAMON/FOIE 30u x110 gr</t>
+  </si>
+  <si>
+    <t>11080 =ALCACHOFAS EN ACEITE 12u x (330</t>
+  </si>
+  <si>
+    <t>11095 =AOVE CON TRUFA NEGRA 12 u x 250 ml</t>
+  </si>
+  <si>
+    <t>LULIÑA</t>
+  </si>
+  <si>
+    <t>MEJILLONES EN ESCABECHE (13-18 PIEZAS) | LULIÑA</t>
+  </si>
+  <si>
+    <t>CHIPIRONES RELLENOS EN SU TINTA | LULIÑA</t>
+  </si>
+  <si>
+    <t>PULPO AHUMADO EN ACEITE DE OLIVA | LULIÑA</t>
+  </si>
+  <si>
+    <t>SARDINILLAS PICANTONAS EN ACEITE DE OLIVA 10-14 PIEZAS | LULIÑA</t>
+  </si>
+  <si>
+    <t>SARDINAS EN ACEITE DE OLIVA 3-4 PIEZAS | LULIÑA</t>
   </si>
 </sst>
 </file>
@@ -3975,16 +4011,16 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <top style="thin">
+        <bottom style="thin">
           <color auto="1"/>
-        </top>
+        </bottom>
       </border>
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
+        <top style="thin">
           <color auto="1"/>
-        </bottom>
+        </top>
       </border>
     </dxf>
     <dxf>
@@ -4030,8 +4066,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9B9C6FA5-7DC8-4D36-BC02-F7E4863161CA}" name="Tabla5" displayName="Tabla5" ref="A1:E1301" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1">
-  <autoFilter ref="A1:E1301" xr:uid="{9B9C6FA5-7DC8-4D36-BC02-F7E4863161CA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9B9C6FA5-7DC8-4D36-BC02-F7E4863161CA}" name="Tabla5" displayName="Tabla5" ref="A1:E1311" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:E1311" xr:uid="{9B9C6FA5-7DC8-4D36-BC02-F7E4863161CA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E1255">
     <sortCondition ref="A1240:A1255"/>
   </sortState>
@@ -4342,7 +4378,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1301"/>
+  <dimension ref="A1:E1311"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.26953125" customWidth="1"/>
@@ -22684,7 +22720,7 @@
       <c r="C1293" t="s">
         <v>45</v>
       </c>
-      <c r="D1293" s="3">
+      <c r="D1293">
         <v>10</v>
       </c>
     </row>
@@ -22698,7 +22734,7 @@
       <c r="C1294" t="s">
         <v>38</v>
       </c>
-      <c r="D1294" s="3">
+      <c r="D1294">
         <v>10</v>
       </c>
     </row>
@@ -22712,7 +22748,7 @@
       <c r="C1295" t="s">
         <v>38</v>
       </c>
-      <c r="D1295" s="3">
+      <c r="D1295">
         <v>10</v>
       </c>
     </row>
@@ -22726,11 +22762,11 @@
       <c r="C1296" t="s">
         <v>108</v>
       </c>
-      <c r="D1296" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="1297" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D1296">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1297" t="s">
         <v>1284</v>
       </c>
@@ -22740,11 +22776,11 @@
       <c r="C1297" t="s">
         <v>38</v>
       </c>
-      <c r="D1297" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="1298" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D1297">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1298" t="s">
         <v>1284</v>
       </c>
@@ -22754,11 +22790,11 @@
       <c r="C1298" t="s">
         <v>45</v>
       </c>
-      <c r="D1298" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="1299" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D1298">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1299" t="s">
         <v>1284</v>
       </c>
@@ -22768,11 +22804,11 @@
       <c r="C1299" t="s">
         <v>45</v>
       </c>
-      <c r="D1299" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="1300" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D1299">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1300" t="s">
         <v>1284</v>
       </c>
@@ -22782,11 +22818,11 @@
       <c r="C1300" t="s">
         <v>38</v>
       </c>
-      <c r="D1300" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="1301" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D1300">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1301" t="s">
         <v>1284</v>
       </c>
@@ -22796,8 +22832,178 @@
       <c r="C1301" t="s">
         <v>108</v>
       </c>
-      <c r="D1301" s="3">
-        <v>10</v>
+      <c r="D1301">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1302" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1302" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1302" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C1302" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1302" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1302">
+        <v>10025</v>
+      </c>
+    </row>
+    <row r="1303" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1303" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1303" t="s">
+        <v>1286</v>
+      </c>
+      <c r="C1303" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1303" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1303">
+        <v>10094</v>
+      </c>
+    </row>
+    <row r="1304" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1304" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1304" t="s">
+        <v>1288</v>
+      </c>
+      <c r="C1304" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1304" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1304">
+        <v>10364</v>
+      </c>
+    </row>
+    <row r="1305" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1305" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1305" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C1305" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1305" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1305">
+        <v>10062</v>
+      </c>
+    </row>
+    <row r="1306" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1306" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1306" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C1306" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1306" s="3">
+        <v>4</v>
+      </c>
+      <c r="E1306">
+        <v>10365</v>
+      </c>
+    </row>
+    <row r="1307" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1307" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B1307" t="s">
+        <v>1292</v>
+      </c>
+      <c r="C1307" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1307" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1307">
+        <v>10352</v>
+      </c>
+    </row>
+    <row r="1308" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1308" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B1308" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C1308" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1308" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1308">
+        <v>10353</v>
+      </c>
+    </row>
+    <row r="1309" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1309" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B1309" t="s">
+        <v>1294</v>
+      </c>
+      <c r="C1309" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1309" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1309">
+        <v>10354</v>
+      </c>
+    </row>
+    <row r="1310" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1310" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B1310" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C1310" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1310" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1310">
+        <v>10355</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1311" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B1311" t="s">
+        <v>1296</v>
+      </c>
+      <c r="C1311" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1311" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1311">
+        <v>10356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(diccionario): alta ALCAPARRON FRASCO 340 GR EL FARO (CONSERVAS VEGETALES, IVA 10%)
Edición manual 14/05/2026 21:03. Proveedor: GUERRA OLLER FRANCISCO.
Diccionario: 58.934 → 60.383 bytes (Δ +1.449, 1 fila nueva).

Sin impacto en lógica — CategorizarLinea consume el Diccionario en runtime.
Próxima ejecución de Parseo recogerá el artículo automáticamente.

Continuación housekeeping pre-cierre v4.17 → v4.18.
</commit_message>
<xml_diff>
--- a/datos/DiccionarioProveedoresCategoria.xlsx
+++ b/datos/DiccionarioProveedoresCategoria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_ARCHIVOS\TRABAJO\Facturas\gestion-facturas\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D705B248-128C-46CA-B836-EA4074195250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A574EF-87CA-4155-9D64-DAEF767DEB6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Articulos" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="1341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4385" uniqueCount="1343">
   <si>
     <t>PROVEEDOR</t>
   </si>
@@ -4055,6 +4055,12 @@
   </si>
   <si>
     <t>JARDINERIA</t>
+  </si>
+  <si>
+    <t>GENERICO CERVEZA</t>
+  </si>
+  <si>
+    <t>ALCAPARRON FRASCO 340 GR EL FARO</t>
   </si>
 </sst>
 </file>
@@ -4084,27 +4090,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -4124,19 +4115,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
     <dxf>
       <font>
         <b/>
@@ -4180,6 +4168,49 @@
         </top>
       </border>
     </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4194,8 +4225,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1232F1A-7B3D-44BD-AFE8-59BF55A0EBE5}" name="Tabla1" displayName="Tabla1" ref="A1:B166" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
-  <autoFilter ref="A1:B166" xr:uid="{C1232F1A-7B3D-44BD-AFE8-59BF55A0EBE5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2EDE806F-9679-41DD-AB53-FD6AACA57ACE}" name="Tabla2" displayName="Tabla2" ref="A1:E1347" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:E1347" xr:uid="{2EDE806F-9679-41DD-AB53-FD6AACA57ACE}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{8A70A2F2-FFDA-476B-9F68-CB6DB7A8E710}" name="PROVEEDOR"/>
+    <tableColumn id="2" xr3:uid="{1347F9BC-C0EB-43E4-94E2-1D3E470217EB}" name="ARTICULO"/>
+    <tableColumn id="3" xr3:uid="{3EF5C3A0-7FFA-41EE-9600-01370A5FEF75}" name="CATEGORIA"/>
+    <tableColumn id="4" xr3:uid="{99EF0437-2FEB-4212-9C90-4921F085BB42}" name="TIPO_IVA"/>
+    <tableColumn id="5" xr3:uid="{BDF3C4CB-7D92-4089-B008-1DA0B27DA391}" name="COD LOYVERSE"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C1232F1A-7B3D-44BD-AFE8-59BF55A0EBE5}" name="Tabla1" displayName="Tabla1" ref="A1:B168" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
+  <autoFilter ref="A1:B168" xr:uid="{C1232F1A-7B3D-44BD-AFE8-59BF55A0EBE5}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="PIMIENTOS PIQUILLO ARTESANOS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D9E76ADF-78E6-4510-B10E-6A251547C131}" name="CATEGORIAS"/>
     <tableColumn id="2" xr3:uid="{C0E9219A-138D-45AC-8930-250F39377B9C}" name="AMBITO"/>
@@ -4489,8 +4540,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1346"/>
+  <dimension ref="A1:E1347"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.26953125" customWidth="1"/>
+    <col min="2" max="2" width="11.1796875" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" customWidth="1"/>
+    <col min="4" max="4" width="10.7265625" customWidth="1"/>
+    <col min="5" max="5" width="15.36328125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -23572,7 +23630,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="1345" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1345" t="s">
         <v>1297</v>
       </c>
@@ -23586,7 +23644,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="1346" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1346" t="s">
         <v>1301</v>
       </c>
@@ -23600,14 +23658,34 @@
         <v>4</v>
       </c>
     </row>
+    <row r="1347" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1347" t="s">
+        <v>1289</v>
+      </c>
+      <c r="B1347" t="s">
+        <v>1342</v>
+      </c>
+      <c r="C1347" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1347">
+        <v>10</v>
+      </c>
+      <c r="E1347">
+        <v>10498</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B166"/>
+  <dimension ref="A1:B168"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.453125" customWidth="1"/>
@@ -23615,14 +23693,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>1302</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1303</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -23630,7 +23708,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -23638,7 +23716,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>455</v>
       </c>
@@ -23646,7 +23724,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -23654,7 +23732,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>120</v>
       </c>
@@ -23662,7 +23740,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>1306</v>
       </c>
@@ -23670,7 +23748,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>1307</v>
       </c>
@@ -23678,7 +23756,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>1308</v>
       </c>
@@ -23686,7 +23764,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>138</v>
       </c>
@@ -23694,7 +23772,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>631</v>
       </c>
@@ -23702,7 +23780,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>140</v>
       </c>
@@ -23710,7 +23788,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>144</v>
       </c>
@@ -23718,7 +23796,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -23726,7 +23804,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>1309</v>
       </c>
@@ -23734,7 +23812,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>1310</v>
       </c>
@@ -23742,7 +23820,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>1147</v>
       </c>
@@ -23750,7 +23828,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>162</v>
       </c>
@@ -23758,7 +23836,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>349</v>
       </c>
@@ -23766,7 +23844,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>1311</v>
       </c>
@@ -23774,7 +23852,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>1312</v>
       </c>
@@ -23782,7 +23860,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>168</v>
       </c>
@@ -23790,7 +23868,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>788</v>
       </c>
@@ -23798,7 +23876,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -23806,7 +23884,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -23814,7 +23892,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>362</v>
       </c>
@@ -23822,7 +23900,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>351</v>
       </c>
@@ -23830,7 +23908,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>360</v>
       </c>
@@ -23838,7 +23916,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>551</v>
       </c>
@@ -23846,7 +23924,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>1107</v>
       </c>
@@ -23854,7 +23932,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>1313</v>
       </c>
@@ -23862,7 +23940,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>398</v>
       </c>
@@ -23870,7 +23948,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>371</v>
       </c>
@@ -23878,7 +23956,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>84</v>
       </c>
@@ -23886,7 +23964,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>87</v>
       </c>
@@ -23894,7 +23972,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>17</v>
       </c>
@@ -23902,7 +23980,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>1314</v>
       </c>
@@ -23910,7 +23988,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>697</v>
       </c>
@@ -23918,7 +23996,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>1315</v>
       </c>
@@ -23926,7 +24004,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>353</v>
       </c>
@@ -23934,7 +24012,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>76</v>
       </c>
@@ -23942,7 +24020,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>94</v>
       </c>
@@ -23950,7 +24028,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>1316</v>
       </c>
@@ -23958,7 +24036,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>1105</v>
       </c>
@@ -23966,7 +24044,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>186</v>
       </c>
@@ -23974,7 +24052,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>1318</v>
       </c>
@@ -23982,7 +24060,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>1319</v>
       </c>
@@ -23990,7 +24068,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>1320</v>
       </c>
@@ -23998,7 +24076,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>129</v>
       </c>
@@ -24006,7 +24084,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>200</v>
       </c>
@@ -24014,7 +24092,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>142</v>
       </c>
@@ -24022,7 +24100,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>70</v>
       </c>
@@ -24030,7 +24108,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>127</v>
       </c>
@@ -24038,7 +24116,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>54</v>
       </c>
@@ -24046,7 +24124,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>1321</v>
       </c>
@@ -24054,7 +24132,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>785</v>
       </c>
@@ -24062,7 +24140,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>699</v>
       </c>
@@ -24070,7 +24148,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>816</v>
       </c>
@@ -24078,7 +24156,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>818</v>
       </c>
@@ -24086,7 +24164,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>831</v>
       </c>
@@ -24094,7 +24172,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>24</v>
       </c>
@@ -24102,7 +24180,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>30</v>
       </c>
@@ -24110,7 +24188,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>219</v>
       </c>
@@ -24118,7 +24196,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>692</v>
       </c>
@@ -24126,7 +24204,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>63</v>
       </c>
@@ -24134,7 +24212,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>34</v>
       </c>
@@ -24142,7 +24220,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>1322</v>
       </c>
@@ -24150,7 +24228,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>32</v>
       </c>
@@ -24158,7 +24236,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>36</v>
       </c>
@@ -24166,7 +24244,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>1323</v>
       </c>
@@ -24174,7 +24252,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>917</v>
       </c>
@@ -24182,7 +24260,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>862</v>
       </c>
@@ -24190,7 +24268,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>920</v>
       </c>
@@ -24198,7 +24276,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -24206,7 +24284,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>444</v>
       </c>
@@ -24214,7 +24292,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>48</v>
       </c>
@@ -24222,7 +24300,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>1324</v>
       </c>
@@ -24230,7 +24308,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>797</v>
       </c>
@@ -24238,7 +24316,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>1325</v>
       </c>
@@ -24246,7 +24324,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>355</v>
       </c>
@@ -24254,7 +24332,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>810</v>
       </c>
@@ -24262,7 +24340,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>151</v>
       </c>
@@ -24270,7 +24348,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>40</v>
       </c>
@@ -24278,7 +24356,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>320</v>
       </c>
@@ -24286,7 +24364,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>188</v>
       </c>
@@ -24294,7 +24372,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>250</v>
       </c>
@@ -24302,7 +24380,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>26</v>
       </c>
@@ -24310,7 +24388,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>644</v>
       </c>
@@ -24326,7 +24404,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>646</v>
       </c>
@@ -24334,7 +24412,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>1300</v>
       </c>
@@ -24342,7 +24420,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>412</v>
       </c>
@@ -24350,7 +24428,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>263</v>
       </c>
@@ -24358,7 +24436,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>410</v>
       </c>
@@ -24366,7 +24444,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>440</v>
       </c>
@@ -24374,7 +24452,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>446</v>
       </c>
@@ -24382,7 +24460,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>1326</v>
       </c>
@@ -24390,7 +24468,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>783</v>
       </c>
@@ -24398,7 +24476,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>787</v>
       </c>
@@ -24406,7 +24484,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>794</v>
       </c>
@@ -24414,7 +24492,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>1327</v>
       </c>
@@ -24422,7 +24500,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>814</v>
       </c>
@@ -24430,7 +24508,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>122</v>
       </c>
@@ -24438,7 +24516,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>612</v>
       </c>
@@ -24446,7 +24524,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>947</v>
       </c>
@@ -24454,7 +24532,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>285</v>
       </c>
@@ -24462,7 +24540,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>481</v>
       </c>
@@ -24470,7 +24548,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>1328</v>
       </c>
@@ -24478,7 +24556,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>1329</v>
       </c>
@@ -24486,7 +24564,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>1330</v>
       </c>
@@ -24494,7 +24572,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>694</v>
       </c>
@@ -24502,7 +24580,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>179</v>
       </c>
@@ -24510,7 +24588,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>182</v>
       </c>
@@ -24518,7 +24596,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>548</v>
       </c>
@@ -24526,7 +24604,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>448</v>
       </c>
@@ -24534,7 +24612,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>52</v>
       </c>
@@ -24542,7 +24620,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>367</v>
       </c>
@@ -24550,7 +24628,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>332</v>
       </c>
@@ -24558,7 +24636,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>406</v>
       </c>
@@ -24566,7 +24644,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>824</v>
       </c>
@@ -24574,7 +24652,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>776</v>
       </c>
@@ -24582,7 +24660,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>404</v>
       </c>
@@ -24590,7 +24668,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>822</v>
       </c>
@@ -24598,7 +24676,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>826</v>
       </c>
@@ -24606,7 +24684,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>56</v>
       </c>
@@ -24614,7 +24692,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>341</v>
       </c>
@@ -24622,7 +24700,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>779</v>
       </c>
@@ -24630,7 +24708,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>59</v>
       </c>
@@ -24638,7 +24716,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>781</v>
       </c>
@@ -24646,7 +24724,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>773</v>
       </c>
@@ -24654,7 +24732,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>431</v>
       </c>
@@ -24662,7 +24740,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>806</v>
       </c>
@@ -24670,7 +24748,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>854</v>
       </c>
@@ -24678,7 +24756,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>154</v>
       </c>
@@ -24686,7 +24764,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>838</v>
       </c>
@@ -24694,7 +24772,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>770</v>
       </c>
@@ -24702,7 +24780,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>1220</v>
       </c>
@@ -24710,7 +24788,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>334</v>
       </c>
@@ -24718,7 +24796,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>1170</v>
       </c>
@@ -24726,7 +24804,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>1331</v>
       </c>
@@ -24734,7 +24812,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>1263</v>
       </c>
@@ -24742,7 +24820,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>7</v>
       </c>
@@ -24750,7 +24828,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>808</v>
       </c>
@@ -24758,7 +24836,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>791</v>
       </c>
@@ -24766,7 +24844,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>1332</v>
       </c>
@@ -24774,7 +24852,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>799</v>
       </c>
@@ -24782,7 +24860,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>801</v>
       </c>
@@ -24790,7 +24868,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>45</v>
       </c>
@@ -24798,7 +24876,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>305</v>
       </c>
@@ -24806,7 +24884,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>226</v>
       </c>
@@ -24814,7 +24892,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>1333</v>
       </c>
@@ -24822,7 +24900,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>856</v>
       </c>
@@ -24830,7 +24908,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>858</v>
       </c>
@@ -24838,7 +24916,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>1265</v>
       </c>
@@ -24846,7 +24924,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>1260</v>
       </c>
@@ -24854,7 +24932,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>1334</v>
       </c>
@@ -24862,7 +24940,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>1335</v>
       </c>
@@ -24870,7 +24948,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>1336</v>
       </c>
@@ -24878,7 +24956,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>1337</v>
       </c>
@@ -24886,7 +24964,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>1338</v>
       </c>
@@ -24894,7 +24972,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>1339</v>
       </c>
@@ -24902,7 +24980,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>1281</v>
       </c>
@@ -24910,7 +24988,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>1340</v>
       </c>
@@ -24918,7 +24996,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>1267</v>
       </c>
@@ -24926,7 +25004,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>504</v>
       </c>
@@ -24934,11 +25012,20 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>659</v>
       </c>
       <c r="B166" t="s">
+        <v>1304</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="168" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A168" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B168" t="s">
         <v>1304</v>
       </c>
     </row>

</xml_diff>